<commit_message>
Mise à jour excel
</commit_message>
<xml_diff>
--- a/data/test/data.xlsx
+++ b/data/test/data.xlsx
@@ -8,7 +8,7 @@
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="welcome_front" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="test" sheetId="1" state="visible" r:id="rId3"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -140,7 +140,7 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -334,11 +334,11 @@
   <dimension ref="A1:AMJ124"/>
   <sheetFormatPr defaultColWidth="12.390625" defaultRowHeight="21.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="8.62"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="12.23"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="14.46"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="10.15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="25.18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="21.97"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="18.64"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="17.11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="16.27"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="25.45"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="15.85"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="14.6"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1024" min="1023" style="1" width="11.52"/>
@@ -386,7 +386,7 @@
       </c>
       <c r="E2" s="1" t="str">
         <f aca="true">"test" &amp; ROW(E1) &amp; "-" &amp; TEXT(TODAY(),"aaaa-mm-jj") &amp; "@test.com"</f>
-        <v>test1-2024-10-24@test.com</v>
+        <v>test1-2024-11-04@test.com</v>
       </c>
       <c r="F2" s="1" t="n">
         <v>611223344</v>
@@ -413,7 +413,7 @@
       </c>
       <c r="E3" s="1" t="str">
         <f aca="true">"test" &amp; ROW(E2) &amp; "-" &amp; TEXT(TODAY(),"aaaa-mm-jj") &amp; "@test.com"</f>
-        <v>test2-2024-10-24@test.com</v>
+        <v>test2-2024-11-04@test.com</v>
       </c>
       <c r="F3" s="1" t="n">
         <v>622334455</v>
@@ -440,7 +440,7 @@
       </c>
       <c r="E4" s="1" t="str">
         <f aca="true">"test" &amp; ROW(E3) &amp; "-" &amp; TEXT(TODAY(),"aaaa-mm-jj") &amp; "@test.com"</f>
-        <v>test3-2024-10-24@test.com</v>
+        <v>test3-2024-11-04@test.com</v>
       </c>
       <c r="F4" s="1" t="n">
         <v>633445566</v>

</xml_diff>